<commit_message>
Double-check Dafy : croisement de dispo Motoblouz x Dafy
- Surveillance correcte des 68 casques (dédup par URL, coloris distingués par
  leurs vraies couleurs au lieu du nom court qui fusionnait des déclinaisons)
- Scraping des casques Shoei sur Dafy (catégorie de contrôle configurable)
- Matching strict gamme + série exacte (graphiques) ou uni<->uni (coloris simples)
  pour éviter les faux positifs ; cas incertains marqués 'non vérifié'
- Rapport : chaque taille en rupture indique le statut Dafy (confirmé / dispo ailleurs)
  + résumé du croisement en en-tête
- Tests unitaires du matching
</commit_message>
<xml_diff>
--- a/reports/rapport_2026-06-08.xlsx
+++ b/reports/rapport_2026-06-08.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O53"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ABIDING</t>
+          <t>ABIDING · Gris/Noir/Jaune</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>BLAST</t>
+          <t>BLAST · Blanc/Bleu/Noir</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MM93 COLLECTION CLASSIC</t>
+          <t>MM93 COLLECTION CLASSIC · Noir/Blanc</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -803,14 +803,10 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GRIP MM93</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>759 €</t>
-        </is>
-      </c>
+          <t>DISCIPLINE · Noir/Rouge</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Rupture</t>
@@ -821,14 +817,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -858,7 +854,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-grip-mm93-260824.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-discipline-319708.html</t>
         </is>
       </c>
     </row>
@@ -875,13 +871,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HORNET ADV 06</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>GRIP MM93 · Noir/Rouge</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>599 €</t>
+          <t>759 €</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -894,9 +894,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -904,24 +904,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-hornet-adv-06-368406.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-grip-mm93-260824.html</t>
         </is>
       </c>
     </row>
@@ -948,19 +948,15 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>HORNET ADV 06</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>INVIGORATE</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>729 €</t>
-        </is>
-      </c>
+          <t>HIKE · Noir/Orange</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Rupture</t>
@@ -981,24 +977,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1008,7 +1004,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-hornet-adv-06-invigorate-368407.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-hike-261792.html</t>
         </is>
       </c>
     </row>
@@ -1025,19 +1021,15 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>J.O2</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AVENTURE</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>469 €</t>
-        </is>
-      </c>
+          <t>MIKE · Bleu</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Rupture</t>
@@ -1085,7 +1077,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-aventure-334326.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-mike-334285.html</t>
         </is>
       </c>
     </row>
@@ -1102,19 +1094,15 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>J.O2</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CANDY</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>399 €</t>
-        </is>
-      </c>
+          <t>MIKE · Gris/Vert</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Rupture</t>
@@ -1162,7 +1150,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-candy-334328.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-mike-334286.html</t>
         </is>
       </c>
     </row>
@@ -1179,17 +1167,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>J.O2</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CROSS LOGO 2</t>
+          <t>MIKE · Jaune/Blanc</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>469 €</t>
+          <t>729 €</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1202,9 +1190,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1239,7 +1227,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-cross-logo-2-334327.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-mike-334283.html</t>
         </is>
       </c>
     </row>
@@ -1256,32 +1244,28 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FEARLESS</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>599 €</t>
-        </is>
-      </c>
+          <t>SCENARIO · Noir/Jaune</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1289,19 +1273,19 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
@@ -1316,7 +1300,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-fearless-334269.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-scenario-241426.html</t>
         </is>
       </c>
     </row>
@@ -1333,17 +1317,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>HORNET ADV 06</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>H-MOBILITY ZAKU</t>
+          <t>Gris/Blanc/Noir</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>639 €</t>
+          <t>599 €</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1351,9 +1335,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1376,14 +1360,14 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1393,7 +1377,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-h-mobility-zaku-338767.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-hornet-adv-06-368406.html</t>
         </is>
       </c>
     </row>
@@ -1410,23 +1394,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>HORNET ADV 06</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IDEOGRAPH</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>INVIGORATE · Noir/Vert/Blanc</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>729 €</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1449,14 +1437,14 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1466,7 +1454,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ideograph-344895.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-hornet-adv-06-invigorate-368407.html</t>
         </is>
       </c>
     </row>
@@ -1483,17 +1471,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>J.O2</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MS-04 RAMBA RAL’S BUGU</t>
+          <t>AVENTURE · Bleu/Noir/Gris</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>639 €</t>
+          <t>469 €</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1501,9 +1489,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1516,14 +1504,14 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1543,7 +1531,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ms-04-ramba-ral-s-bugu-338766.html</t>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-aventure-334326.html</t>
         </is>
       </c>
     </row>
@@ -1560,17 +1548,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>J.O2</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MS-05 ZAKU I</t>
+          <t>CANDY · Bleu/Rouge/Gris</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>639 €</t>
+          <t>399 €</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1578,9 +1566,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -1620,7 +1608,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ms-05-zaku-i-338768.html</t>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-candy-334325.html</t>
         </is>
       </c>
     </row>
@@ -1637,17 +1625,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>J.O2</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ORIGAMI2</t>
+          <t>CANDY · Gris/Marron/Noir</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>599 €</t>
+          <t>399 €</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1655,9 +1643,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1697,7 +1685,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-origami2-338320.html</t>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-candy-334328.html</t>
         </is>
       </c>
     </row>
@@ -1714,17 +1702,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>X-SPR PRO</t>
+          <t>J.O2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>GARDNER</t>
+          <t>CROSS LOGO 2 · Blanc/Noir</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>949 €</t>
+          <t>469 €</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1737,9 +1725,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1747,24 +1735,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="M17" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -1774,7 +1762,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-gardner-334263.html</t>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-cross-logo-2-334327.html</t>
         </is>
       </c>
     </row>
@@ -1791,17 +1779,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>X-SPR PRO</t>
+          <t>NXR2</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MARQUEZ MOTEGI 5</t>
+          <t>FEARLESS · Noir/Jaune/Blanc</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>949 €</t>
+          <t>599 €</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1809,9 +1797,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1839,9 +1827,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1851,7 +1839,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-marquez-motegi-5-359684.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-fearless-334269.html</t>
         </is>
       </c>
     </row>
@@ -1868,17 +1856,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>X-SPR PRO</t>
+          <t>NXR2</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TOPRAK</t>
+          <t>H-MOBILITY ZAKU · Violet</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>949 €</t>
+          <t>639 €</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1886,9 +1874,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1928,7 +1916,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-toprak-359683.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-h-mobility-zaku-338767.html</t>
         </is>
       </c>
     </row>
@@ -1945,23 +1933,23 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>X-SPR PRO 02 FIM2</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>859 €</t>
-        </is>
-      </c>
+          <t>NXR2</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IDEOGRAPH · Noir/Blanc</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>Rupture</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -2001,7 +1989,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-02-fim2-368405.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ideograph-344895.html</t>
         </is>
       </c>
     </row>
@@ -2018,24 +2006,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GLAMSTER 06</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+          <t>NXR2</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MS-04 RAMBA RAL’S BUGU · Noir/Bleu/Blanc</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>639 €</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Partiel</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -2043,24 +2039,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
-        </is>
-      </c>
-      <c r="M21" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -2070,7 +2066,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-glamster-06-385075.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ms-04-ramba-ral-s-bugu-338766.html</t>
         </is>
       </c>
     </row>
@@ -2087,32 +2083,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GLAMSTER 06</t>
+          <t>NXR2</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>HEIWA MOTORCYCLE</t>
+          <t>MS-05 ZAKU I · Noir/Gris</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>599 €</t>
+          <t>639 €</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Partiel</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -2120,19 +2116,19 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -2147,7 +2143,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-glamster-06-heiwa-motorcycle-261817.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ms-05-zaku-i-338768.html</t>
         </is>
       </c>
     </row>
@@ -2164,12 +2160,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GLAMSTER 06</t>
+          <t>NXR2</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>NEIGHBORHOOD x DEATH SPRAY CUSTOM</t>
+          <t>ORIGAMI2 · Noir/Blanc</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2179,17 +2175,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Partiel</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -2207,14 +2203,14 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
-        </is>
-      </c>
-      <c r="M23" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -2224,7 +2220,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-glamster-06-neighborhood-x-death-spray-custom-236861.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-origami2-338320.html</t>
         </is>
       </c>
     </row>
@@ -2241,18 +2237,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GT-AIR 3</t>
+          <t>X-SPR PRO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DISCIPLINE</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
+          <t>GARDNER · Bleu</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>949 €</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2265,9 +2265,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2280,14 +2280,14 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-discipline-319709.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-gardner-334263.html</t>
         </is>
       </c>
     </row>
@@ -2314,18 +2314,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GT-AIR 3</t>
+          <t>X-SPR PRO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>HIKE</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>MARQUEZ MOTEGI 5 · Noir/Gris</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>949 €</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2333,9 +2337,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -2353,9 +2357,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
@@ -2370,7 +2374,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-hike-261793.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-marquez-motegi-5-359684.html</t>
         </is>
       </c>
     </row>
@@ -2387,22 +2391,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GT-AIR 3</t>
+          <t>X-SPR PRO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>LILT</t>
+          <t>TOPRAK · Gris/Bleu</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>729 €</t>
+          <t>949 €</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2420,24 +2424,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="M26" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -2447,7 +2451,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-lilt-261794.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-toprak-359683.html</t>
         </is>
       </c>
     </row>
@@ -2464,18 +2468,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GT-AIR 3</t>
+          <t>X-SPR PRO 02 FIM2</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>REALM</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
+          <t>Noir/Blanc</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>859 €</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2493,14 +2501,14 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
@@ -2508,9 +2516,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -2520,7 +2528,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-realm-319707.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-02-fim2-368405.html</t>
         </is>
       </c>
     </row>
@@ -2537,19 +2545,15 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GT-AIR 3</t>
+          <t>GLAMSTER 06</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SCENARIO</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>729 €</t>
-        </is>
-      </c>
+          <t>Gris</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Partiel</t>
@@ -2560,9 +2564,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -2570,24 +2574,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="M28" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
@@ -2597,7 +2601,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-scenario-241425.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-glamster-06-385075.html</t>
         </is>
       </c>
     </row>
@@ -2614,17 +2618,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
+          <t>GLAMSTER 06</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>INSPIRED</t>
+          <t>HEIWA MOTORCYCLE · Noir</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>649 €</t>
+          <t>599 €</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2637,9 +2641,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -2647,24 +2651,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L29" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M29" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -2674,7 +2678,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-inspired-272896.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-glamster-06-heiwa-motorcycle-261817.html</t>
         </is>
       </c>
     </row>
@@ -2691,17 +2695,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
+          <t>GLAMSTER 06</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>WHIZZY</t>
+          <t>NEIGHBORHOOD x DEATH SPRAY CUSTOM · Noir/Blanc</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>649 €</t>
+          <t>599 €</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2714,9 +2718,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -2734,9 +2738,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
@@ -2751,7 +2755,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-whizzy-261816.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-glamster-06-neighborhood-x-death-spray-custom-236861.html</t>
         </is>
       </c>
     </row>
@@ -2768,48 +2772,48 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>NXR2</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>449,10 €</t>
-        </is>
-      </c>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>DISCIPLINE · Noir/Bleu</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -2824,7 +2828,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-269497.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-discipline-319709.html</t>
         </is>
       </c>
     </row>
@@ -2841,27 +2845,23 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>BEAUT</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>599 €</t>
-        </is>
-      </c>
+          <t>HIKE · Noir/Jaune</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2884,14 +2884,14 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M32" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-beaut-261797.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-hike-261793.html</t>
         </is>
       </c>
     </row>
@@ -2918,23 +2918,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CANDY MATT</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
+          <t>LILT · Bleu/Blanc</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>729 €</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -2947,34 +2951,34 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L33" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="N33" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-candy-matt-241165.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-lilt-261794.html</t>
         </is>
       </c>
     </row>
@@ -2991,27 +2995,23 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CAPRICCIO</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>599 €</t>
-        </is>
-      </c>
+          <t>REALM · Noir/Rouge</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -3039,9 +3039,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="M34" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-capriccio-236862.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-realm-319707.html</t>
         </is>
       </c>
     </row>
@@ -3068,23 +3068,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FORTRESS</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
+          <t>SCENARIO · Noir/Blanc</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>729 €</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -3107,9 +3111,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="L35" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
@@ -3124,7 +3128,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-fortress-268973.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-scenario-241425.html</t>
         </is>
       </c>
     </row>
@@ -3141,37 +3145,33 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>J-CRUISE 3</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>HATSUNE MIKU</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>639 €</t>
-        </is>
-      </c>
+          <t>Bleu</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-hatsune-miku-334273.html</t>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-401230.html</t>
         </is>
       </c>
     </row>
@@ -3218,17 +3218,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>J-CRUISE 3</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>KNEE DOWN</t>
+          <t>INSPIRED · Noir/Rouge</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>599 €</t>
+          <t>649 €</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3236,14 +3236,14 @@
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -3251,24 +3251,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 17/06/26</t>
-        </is>
-      </c>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 17/06/26</t>
-        </is>
-      </c>
-      <c r="L37" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 17/06/26</t>
-        </is>
-      </c>
-      <c r="M37" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 17/06/26</t>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-knee-down-272116.html</t>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-inspired-272896.html</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>J-CRUISE 3</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>MS-06C-6 ZAKU II</t>
+          <t>WHIZZY · Noir/Rouge/Blanc</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>639 €</t>
+          <t>649 €</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3313,9 +3313,9 @@
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -3343,9 +3343,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ms-06c-6-zaku-ii-334271.html</t>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-whizzy-261816.html</t>
         </is>
       </c>
     </row>
@@ -3377,12 +3377,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>PLAIN</t>
+          <t>BEAUT · Noir/Rouge/Blanc</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>479 €</t>
+          <t>599 €</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3395,9 +3395,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -3420,19 +3420,19 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="M39" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="N39" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-plain-207262.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-beaut-261797.html</t>
         </is>
       </c>
     </row>
@@ -3454,12 +3454,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>RX-78-02 GUNDAM</t>
+          <t>CANDY MATT · Bleu</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>639 €</t>
+          <t>499 €</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3472,9 +3472,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -3482,19 +3482,19 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>Réappro 09/06/26</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="L40" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-rx-78-02-gundam-334272.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-candy-matt-208567.html</t>
         </is>
       </c>
     </row>
@@ -3526,23 +3526,23 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>X-SPR PRO</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>719,10 €</t>
-        </is>
-      </c>
+          <t>NXR2</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>CANDY MATT · Noir</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -3555,34 +3555,34 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J41" s="5" t="inlineStr">
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
         <is>
           <t>Réappro 09/06/26</t>
         </is>
       </c>
-      <c r="K41" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L41" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M41" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-220680.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-candy-matt-241165.html</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3599,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>X-SPR PRO</t>
+          <t>NXR2</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>DIGGIA 2</t>
+          <t>CAPRICCIO · Noir/Violet/Blanc</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>949 €</t>
+          <t>599 €</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3617,9 +3617,9 @@
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -3632,14 +3632,14 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
@@ -3647,9 +3647,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="M42" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-diggia-2-261789.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-capriccio-236862.html</t>
         </is>
       </c>
     </row>
@@ -3676,28 +3676,28 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>X-SPR PRO ALEX MARQUEZ 73 V2</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>949 €</t>
-        </is>
-      </c>
+          <t>NXR2</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>FORTRESS · Blanc/Gris</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -3705,9 +3705,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
@@ -3715,9 +3715,9 @@
           <t>Rupture</t>
         </is>
       </c>
-      <c r="L43" s="4" t="inlineStr">
-        <is>
-          <t>Rupture</t>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-alex-marquez-73-v2-227002.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-fortress-268973.html</t>
         </is>
       </c>
     </row>
@@ -3749,19 +3749,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GT-AIR 3</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+          <t>NXR2</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Gris</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>449,10 €</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -3784,9 +3792,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L44" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr">
@@ -3801,7 +3809,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-269203.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-269497.html</t>
         </is>
       </c>
     </row>
@@ -3818,37 +3826,37 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>GT-AIR 3</t>
+          <t>NXR2</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>AGILITY</t>
+          <t>HATSUNE MIKU · Bleu</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>729 €</t>
+          <t>639 €</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="I45" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
@@ -3866,9 +3874,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="M45" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -3878,7 +3886,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-agility-338323.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-hatsune-miku-334273.html</t>
         </is>
       </c>
     </row>
@@ -3895,28 +3903,32 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>GT-AIR 3</t>
+          <t>NXR2</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>MIKE</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr"/>
+          <t>KNEE DOWN · Noir/Rouge</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>599 €</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -3924,24 +3936,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J46" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K46" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L46" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M46" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 17/06/26</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 17/06/26</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 17/06/26</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 17/06/26</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
@@ -3951,7 +3963,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-mike-334284.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-knee-down-272116.html</t>
         </is>
       </c>
     </row>
@@ -3968,19 +3980,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
+          <t>NXR2</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>MS-06C-6 ZAKU II · Noir/Vert</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>639 €</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
@@ -4020,7 +4040,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-334953.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ms-06c-6-zaku-ii-334271.html</t>
         </is>
       </c>
     </row>
@@ -4037,27 +4057,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>J.O2</t>
+          <t>NXR2</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PLAIN</t>
+          <t>PLAIN · Noir/Blanc</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>399 €</t>
+          <t>479 €</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -4090,14 +4110,14 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="N48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="N48" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-plain-334324.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-plain-207262.html</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4139,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>MS-06S CHAR’S ZAKU II</t>
+          <t>RX-78-02 GUNDAM · Blanc/Bleu</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4129,12 +4149,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -4147,24 +4167,24 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J49" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K49" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L49" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M49" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
@@ -4174,7 +4194,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ms-06s-char-s-zaku-ii-334270.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-rx-78-02-gundam-334272.html</t>
         </is>
       </c>
     </row>
@@ -4191,27 +4211,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NXR2</t>
+          <t>X-SPR PRO</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>SHINE</t>
+          <t>DIGGIA 2 · Noir/Rouge</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>499 €</t>
+          <t>949 €</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
@@ -4239,9 +4259,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="M50" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -4251,7 +4271,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-shine-207263.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-diggia-2-261789.html</t>
         </is>
       </c>
     </row>
@@ -4273,17 +4293,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>A.MARQUEZ  73 V3</t>
+          <t>Noir/Blanc</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>949 €</t>
+          <t>719,10 €</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Complet</t>
+          <t>Partiel</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -4301,9 +4321,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J51" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 09/06/26</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
@@ -4328,7 +4348,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-a-marquez-73-v3-398626.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-220680.html</t>
         </is>
       </c>
     </row>
@@ -4345,12 +4365,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>X-SPR PRO</t>
+          <t>X-SPR PRO ALEX MARQUEZ 73 V2</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>MARC MARQUEZ MOTEGI 5</t>
+          <t>Bleu/Blanc</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4360,7 +4380,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Complet</t>
+          <t>Partiel</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -4383,19 +4403,19 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="K52" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L52" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M52" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M52" s="4" t="inlineStr">
+        <is>
+          <t>Rupture</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
@@ -4405,7 +4425,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-marc-marquez-motegi-5-271767.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-alex-marquez-73-v2-227002.html</t>
         </is>
       </c>
     </row>
@@ -4422,65 +4442,1273 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
+          <t>GLAMSTER 06</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Noir/Bleu/Blanc</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>469 €</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-glamster-06-220714.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>AGILITY · Noir/Rouge/Blanc</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>729 €</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-agility-338323.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-269204.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Gris</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-269496.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Jaune/Gris/Bleu</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>629 €</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-236860.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>MIKE · Blanc/Noir</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-mike-334284.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-269203.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-334952.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Gris</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-269498.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M62" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-334953.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Noir/Blanc/Gris</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M63" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-261815.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>J.O2</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>PLAIN · Noir/Blanc</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>399 €</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M64" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-o2-plain-334324.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>NXR2</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>MS-06S CHAR’S ZAKU II · Noir/Rouge</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>639 €</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-ms-06s-char-s-zaku-ii-334270.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>NXR2</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>SHINE · Rouge/Gris</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>499 €</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M66" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-nxr2-shine-207263.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
           <t>X-SPR PRO</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>VALION</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>A.MARQUEZ  73 V3 · Noir/Bleu</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>949 €</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M67" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-a-marquez-73-v3-398626.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>X-SPR PRO</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>MARC MARQUEZ MOTEGI 5 · Noir/Rouge</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>949 €</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-marc-marquez-motegi-5-271767.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>X-SPR PRO</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>VALION · Noir/Rouge/Violet</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
         <is>
           <t>899 €</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K53" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L53" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="M53" s="3" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="N53" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
         <is>
           <t>https://www.motoblouz.com/vente-casque-integral-shoei-x-spr-pro-valion-344986.html</t>
         </is>

</xml_diff>

<commit_message>
Éclatement des fiches par coloris (1 résultat par coloris)
- Une fiche Motoblouz peut regrouper plusieurs coloris (ex GT-Air 3 = Bleu mat
  + Gris mat + Jaune sous un seul ID). On groupe désormais les SKU par coloris.
- Finition mat/brillant déduite du nom de coloris de l'image (Matt blue -> Bleu mat),
  liaison couleur FR(SKU) <-> EN(image)
- scrape() renvoie une liste (1 par coloris) ; dédup par (URL, coloris)
- Corrige la perte de coloris comme GT-Air 3 Bleu mat
</commit_message>
<xml_diff>
--- a/reports/rapport_2026-06-08.xlsx
+++ b/reports/rapport_2026-06-08.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -670,10 +670,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Gris</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Bleu mat</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>629 €</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Complet</t>
@@ -711,7 +715,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-269496.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-236860.html</t>
         </is>
       </c>
     </row>
@@ -733,7 +737,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Noir brillant</t>
+          <t>Gris</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -774,7 +778,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-269203.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-269496.html</t>
         </is>
       </c>
     </row>
@@ -796,10 +800,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Noir mat</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>Gris mat</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>629 €</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Complet</t>
@@ -837,7 +845,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-334952.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-236860.html</t>
         </is>
       </c>
     </row>
@@ -854,19 +862,15 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Gris</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>549 €</t>
-        </is>
-      </c>
+          <t>Noir brillant</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Complet</t>
@@ -904,7 +908,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-269498.html</t>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-269203.html</t>
         </is>
       </c>
     </row>
@@ -921,7 +925,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -966,6 +970,337 @@
         </is>
       </c>
       <c r="M8" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-integral-shoei-gt-air-3-334952.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-261815.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Gris</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-261815.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Gris</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-269498.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Noir brillant</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-261815.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Shoei</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Noir mat</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>https://www.motoblouz.com/vente-casque-jet-shoei-j-cruise-3-334953.html</t>
         </is>

</xml_diff>

<commit_message>
Affichage du nom de coloris précis (Gris Chalk, Gris Basalt, Bleu mat...)
- Extrait le qualificatif distinctif du nom de coloris de l'image
- Distingue les coloris de même couleur de base (2 gris différents)
</commit_message>
<xml_diff>
--- a/reports/rapport_2026-06-08.xlsx
+++ b/reports/rapport_2026-06-08.xlsx
@@ -836,7 +836,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 21:02   ·   12 casques   ·   🟢 11 complets   🟡 1 partiels   🔴 0 ruptures</t>
+          <t>08/06/2026 21:11   ·   12 casques   ·   🟢 11 complets   🟡 1 partiels   🔴 0 ruptures</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Gris</t>
+          <t>Gris Chalk</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr"/>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Gris mat</t>
+          <t>Gris Deep mat</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Gris</t>
+          <t>Gris Basalt</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Gris</t>
+          <t>Gris Chalk</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Multi-sites: scraper Motoshopping + colonne Site dans l'Excel
- Scraper Motoshopping (PrestaShop, payload combinationsFromController :
  stock + date de réappro par taille), 1 coloris = 1 URL
- Config multi-sites (Motoblouz + Motoshopping), report groupé par site
- Excel: colonne Site ajoutée
</commit_message>
<xml_diff>
--- a/reports/rapport_2026-06-08.xlsx
+++ b/reports/rapport_2026-06-08.xlsx
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -72,12 +72,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEF3FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -137,6 +142,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -221,7 +229,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>4</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -246,7 +254,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -271,7 +279,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>7</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -296,7 +304,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>8</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -321,7 +329,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>7</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -346,7 +354,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>8</row>
+      <row>12</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -371,7 +379,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -396,7 +404,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>10</row>
+      <row>16</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -421,7 +429,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -446,7 +454,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>12</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -471,7 +479,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -496,7 +504,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>22</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="685800" cy="685800"/>
@@ -809,21 +817,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -836,7 +846,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 21:11   ·   12 casques   ·   🟢 11 complets   🟡 1 partiels   🔴 0 ruptures</t>
+          <t>08/06/2026 21:31   ·   20 casques   ·   🟢 12 complets   🟡 8 partiels   🔴 0 ruptures</t>
         </is>
       </c>
     </row>
@@ -848,55 +858,65 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
           <t>Gamme</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Coloris</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Prix</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>2XL</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Fiche</t>
         </is>
@@ -906,28 +926,32 @@
       <c r="A4" s="4" t="inlineStr"/>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
+          <t>Motoshopping</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Bleu mat</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr">
+          <t>GT-AIR 3</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>479,20 €</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 16/06/26</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -940,17 +964,27 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>Rupture</t>
-        </is>
-      </c>
-      <c r="L4" s="8" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 16/06/26</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 14/07/26</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 16/06/26</t>
+        </is>
+      </c>
+      <c r="N4" s="8" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -960,25 +994,25 @@
       <c r="A5" s="9" t="inlineStr"/>
       <c r="B5" s="9" t="inlineStr">
         <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
           <t>GT-AIR 3</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Blanc</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Dispo</t>
@@ -1004,7 +1038,17 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L5" s="10" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1014,32 +1058,32 @@
       <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>Motoshopping</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>GT-AIR 3</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Bleu mat</t>
-        </is>
-      </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>629 €</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+          <t>Bleu Mat</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>503,20 €</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 07/07/26</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -1047,9 +1091,9 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 13/08/26</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
@@ -1062,7 +1106,17 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 16/06/26</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1072,25 +1126,29 @@
       <c r="A7" s="9" t="inlineStr"/>
       <c r="B7" s="9" t="inlineStr">
         <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
           <t>GT-AIR 3</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Gris Chalk</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Bleu mat</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>629 €</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Dispo</t>
@@ -1116,7 +1174,17 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1126,29 +1194,25 @@
       <c r="A8" s="4" t="inlineStr"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
           <t>GT-AIR 3</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Gris Deep mat</t>
-        </is>
-      </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>629 €</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
+          <t>Gris Chalk</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Dispo</t>
@@ -1174,7 +1238,17 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L8" s="8" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1184,25 +1258,29 @@
       <c r="A9" s="9" t="inlineStr"/>
       <c r="B9" s="9" t="inlineStr">
         <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
           <t>GT-AIR 3</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Noir brillant</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Gris Deep mat</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>629 €</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Dispo</t>
@@ -1228,7 +1306,17 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L9" s="10" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1238,23 +1326,27 @@
       <c r="A10" s="4" t="inlineStr"/>
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>Motoshopping</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
           <t>GT-AIR 3</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Noir mat</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>479,20 €</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Partiel</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -1277,12 +1369,22 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L10" s="8" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 14/07/26</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1292,29 +1394,29 @@
       <c r="A11" s="9" t="inlineStr"/>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
+          <t>Motoshopping</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Blanc</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>549 €</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
+          <t>Noir Mat</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>503,20 €</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Dispo</t>
@@ -1340,7 +1442,17 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L11" s="10" t="inlineStr">
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1350,29 +1462,25 @@
       <c r="A12" s="4" t="inlineStr"/>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
+          <t>Motoblouz</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Gris Basalt</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>549 €</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
+          <t>Noir brillant</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Dispo</t>
@@ -1398,7 +1506,17 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L12" s="8" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1408,29 +1526,25 @@
       <c r="A13" s="9" t="inlineStr"/>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>J-CRUISE 3</t>
+          <t>Motoblouz</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Gris Chalk</t>
+          <t>GT-AIR 3</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>549 €</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
+          <t>Noir mat</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Dispo</t>
@@ -1456,7 +1570,17 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="L13" s="10" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1466,32 +1590,32 @@
       <c r="A14" s="4" t="inlineStr"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Motoshopping</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
           <t>J-CRUISE 3</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Noir brillant</t>
-        </is>
-      </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>549 €</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
+          <t>Blanc</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>439,20 €</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 16/06/26</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -1509,12 +1633,22 @@
           <t>Dispo</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 14/07/26</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 25/08/26</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1524,51 +1658,601 @@
       <c r="A15" s="9" t="inlineStr"/>
       <c r="B15" s="9" t="inlineStr">
         <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
           <t>J-CRUISE 3</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Blanc</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N15" s="10" t="inlineStr">
+        <is>
+          <t>Voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Motoshopping</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Bleu Mat</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>439,20 €</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 16/06/26</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 07/07/26</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>Voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Bleu mat</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
+        <is>
+          <t>Rupture</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N17" s="10" t="inlineStr">
+        <is>
+          <t>Voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Gris Basalt</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>Voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="9" t="inlineStr"/>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Gris Chalk</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N19" s="10" t="inlineStr">
+        <is>
+          <t>Voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Motoshopping</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>439,20 €</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 16/06/26</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 25/08/26</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 14/07/26</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 25/08/26</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>Voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="9" t="inlineStr"/>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Motoshopping</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Noir Mat</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>439,20 €</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 14/07/26</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Réappro 25/08/26</t>
+        </is>
+      </c>
+      <c r="N21" s="10" t="inlineStr">
+        <is>
+          <t>Voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Noir brillant</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>549 €</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>Voir</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="9" t="inlineStr"/>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Motoblouz</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>J-CRUISE 3</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Noir mat</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr"/>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Complet</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>Dispo</t>
-        </is>
-      </c>
-      <c r="L15" s="10" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>Dispo</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="inlineStr">
         <is>
           <t>Voir</t>
         </is>
@@ -1576,24 +2260,32 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>